<commit_message>
Documentação, material de venda, catálogo, kits e relatório de qualidade dos 10 produtos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019swxXDBkedQ8LqP1HPvw4h
</commit_message>
<xml_diff>
--- a/planilhas/financeiro/fluxo-de-caixa/EXEMPLO.xlsx
+++ b/planilhas/financeiro/fluxo-de-caixa/EXEMPLO.xlsx
@@ -1643,8 +1643,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>247650</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>714375</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>

</xml_diff>